<commit_message>
Updated Hotel Booking Dashboard.xlsx
</commit_message>
<xml_diff>
--- a/Project/Hotel Booking Dashboard.xlsx
+++ b/Project/Hotel Booking Dashboard.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B842591-F709-497E-BF98-E8726B83615F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="3" r:id="rId1"/>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="14" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -2845,7 +2845,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2853,17 +2853,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3604,6 +3603,34 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -3637,6 +3664,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-A8FA-4C7B-A290-7F25A57497B3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -3652,6 +3684,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-A8FA-4C7B-A290-7F25A57497B3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -4321,6 +4358,48 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -4354,6 +4433,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-5CB6-464F-8CD9-E6AEBCB8C748}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -4369,6 +4453,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-5CB6-464F-8CD9-E6AEBCB8C748}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -4384,6 +4473,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-5CB6-464F-8CD9-E6AEBCB8C748}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -6758,8 +6852,8 @@
       <xdr:row>21</xdr:row>
       <xdr:rowOff>149222</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="2" name="RoomNo">
@@ -6782,7 +6876,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -6836,8 +6930,8 @@
       <xdr:row>26</xdr:row>
       <xdr:rowOff>53972</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="3" name="PaymentStatus">
@@ -6860,7 +6954,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -10613,344 +10707,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6D12B0F7-3CA9-41E1-BAEE-124641D0366F}" name="PivotTable5" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
-  <location ref="A67:B71" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="251">
-        <item x="70"/>
-        <item x="142"/>
-        <item x="214"/>
-        <item x="5"/>
-        <item x="76"/>
-        <item x="148"/>
-        <item x="220"/>
-        <item x="10"/>
-        <item x="82"/>
-        <item x="154"/>
-        <item x="226"/>
-        <item x="16"/>
-        <item x="88"/>
-        <item x="160"/>
-        <item x="232"/>
-        <item x="22"/>
-        <item x="94"/>
-        <item x="166"/>
-        <item x="238"/>
-        <item x="28"/>
-        <item x="100"/>
-        <item x="172"/>
-        <item x="244"/>
-        <item x="34"/>
-        <item x="106"/>
-        <item x="178"/>
-        <item x="40"/>
-        <item x="112"/>
-        <item x="184"/>
-        <item x="46"/>
-        <item x="118"/>
-        <item x="190"/>
-        <item x="52"/>
-        <item x="124"/>
-        <item x="196"/>
-        <item x="58"/>
-        <item x="130"/>
-        <item x="202"/>
-        <item x="64"/>
-        <item x="136"/>
-        <item x="208"/>
-        <item x="0"/>
-        <item x="71"/>
-        <item x="143"/>
-        <item x="215"/>
-        <item x="6"/>
-        <item x="77"/>
-        <item x="149"/>
-        <item x="221"/>
-        <item x="11"/>
-        <item x="83"/>
-        <item x="155"/>
-        <item x="227"/>
-        <item x="17"/>
-        <item x="89"/>
-        <item x="161"/>
-        <item x="233"/>
-        <item x="23"/>
-        <item x="95"/>
-        <item x="167"/>
-        <item x="239"/>
-        <item x="29"/>
-        <item x="101"/>
-        <item x="173"/>
-        <item x="245"/>
-        <item x="35"/>
-        <item x="107"/>
-        <item x="179"/>
-        <item x="41"/>
-        <item x="113"/>
-        <item x="185"/>
-        <item x="47"/>
-        <item x="119"/>
-        <item x="191"/>
-        <item x="53"/>
-        <item x="125"/>
-        <item x="197"/>
-        <item x="59"/>
-        <item x="131"/>
-        <item x="203"/>
-        <item x="65"/>
-        <item x="137"/>
-        <item x="209"/>
-        <item x="1"/>
-        <item x="72"/>
-        <item x="144"/>
-        <item x="216"/>
-        <item x="7"/>
-        <item x="78"/>
-        <item x="150"/>
-        <item x="222"/>
-        <item x="12"/>
-        <item x="84"/>
-        <item x="156"/>
-        <item x="228"/>
-        <item x="18"/>
-        <item x="90"/>
-        <item x="162"/>
-        <item x="234"/>
-        <item x="24"/>
-        <item x="96"/>
-        <item x="168"/>
-        <item x="240"/>
-        <item x="30"/>
-        <item x="102"/>
-        <item x="174"/>
-        <item x="246"/>
-        <item x="36"/>
-        <item x="108"/>
-        <item x="180"/>
-        <item x="42"/>
-        <item x="114"/>
-        <item x="186"/>
-        <item x="48"/>
-        <item x="120"/>
-        <item x="192"/>
-        <item x="54"/>
-        <item x="126"/>
-        <item x="198"/>
-        <item x="60"/>
-        <item x="132"/>
-        <item x="204"/>
-        <item x="66"/>
-        <item x="138"/>
-        <item x="210"/>
-        <item x="2"/>
-        <item x="73"/>
-        <item x="145"/>
-        <item x="217"/>
-        <item x="8"/>
-        <item x="79"/>
-        <item x="151"/>
-        <item x="223"/>
-        <item x="13"/>
-        <item x="85"/>
-        <item x="157"/>
-        <item x="229"/>
-        <item x="19"/>
-        <item x="91"/>
-        <item x="163"/>
-        <item x="235"/>
-        <item x="25"/>
-        <item x="97"/>
-        <item x="169"/>
-        <item x="241"/>
-        <item x="31"/>
-        <item x="103"/>
-        <item x="175"/>
-        <item x="247"/>
-        <item x="37"/>
-        <item x="109"/>
-        <item x="181"/>
-        <item x="43"/>
-        <item x="115"/>
-        <item x="187"/>
-        <item x="49"/>
-        <item x="121"/>
-        <item x="193"/>
-        <item x="55"/>
-        <item x="127"/>
-        <item x="199"/>
-        <item x="61"/>
-        <item x="133"/>
-        <item x="205"/>
-        <item x="67"/>
-        <item x="139"/>
-        <item x="211"/>
-        <item x="3"/>
-        <item x="74"/>
-        <item x="146"/>
-        <item x="218"/>
-        <item x="9"/>
-        <item x="80"/>
-        <item x="152"/>
-        <item x="224"/>
-        <item x="14"/>
-        <item x="86"/>
-        <item x="158"/>
-        <item x="230"/>
-        <item x="20"/>
-        <item x="92"/>
-        <item x="164"/>
-        <item x="236"/>
-        <item x="26"/>
-        <item x="98"/>
-        <item x="170"/>
-        <item x="242"/>
-        <item x="32"/>
-        <item x="104"/>
-        <item x="176"/>
-        <item x="248"/>
-        <item x="38"/>
-        <item x="110"/>
-        <item x="182"/>
-        <item x="44"/>
-        <item x="116"/>
-        <item x="188"/>
-        <item x="50"/>
-        <item x="122"/>
-        <item x="194"/>
-        <item x="56"/>
-        <item x="128"/>
-        <item x="200"/>
-        <item x="62"/>
-        <item x="134"/>
-        <item x="206"/>
-        <item x="68"/>
-        <item x="140"/>
-        <item x="212"/>
-        <item x="4"/>
-        <item x="75"/>
-        <item x="147"/>
-        <item x="219"/>
-        <item x="81"/>
-        <item x="153"/>
-        <item x="225"/>
-        <item x="15"/>
-        <item x="87"/>
-        <item x="159"/>
-        <item x="231"/>
-        <item x="21"/>
-        <item x="93"/>
-        <item x="165"/>
-        <item x="237"/>
-        <item x="27"/>
-        <item x="99"/>
-        <item x="171"/>
-        <item x="243"/>
-        <item x="33"/>
-        <item x="105"/>
-        <item x="177"/>
-        <item x="249"/>
-        <item x="39"/>
-        <item x="111"/>
-        <item x="183"/>
-        <item x="45"/>
-        <item x="117"/>
-        <item x="189"/>
-        <item x="51"/>
-        <item x="123"/>
-        <item x="195"/>
-        <item x="57"/>
-        <item x="129"/>
-        <item x="201"/>
-        <item x="63"/>
-        <item x="135"/>
-        <item x="207"/>
-        <item x="69"/>
-        <item x="141"/>
-        <item x="213"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="5"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of BookingID" fld="0" subtotal="count" baseField="5" baseItem="1"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="8" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A62FA1C6-6B15-42CF-B8ED-FDCC0FCBC43C}" name="PivotTable4" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A62FA1C6-6B15-42CF-B8ED-FDCC0FCBC43C}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="A43:B50" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField dataField="1" showAll="0"/>
@@ -11288,8 +11045,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4C59890A-608F-4988-B6CF-7001EF1794D9}" name="PivotTable3" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4C59890A-608F-4988-B6CF-7001EF1794D9}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A14:B17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField dataField="1" showAll="0"/>
@@ -11869,8 +11626,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{325A8F64-29CD-470E-9D0F-650C9B1326CD}" name="PivotTable1" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{325A8F64-29CD-470E-9D0F-650C9B1326CD}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -12217,6 +11974,343 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6D12B0F7-3CA9-41E1-BAEE-124641D0366F}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+  <location ref="A67:B71" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="251">
+        <item x="70"/>
+        <item x="142"/>
+        <item x="214"/>
+        <item x="5"/>
+        <item x="76"/>
+        <item x="148"/>
+        <item x="220"/>
+        <item x="10"/>
+        <item x="82"/>
+        <item x="154"/>
+        <item x="226"/>
+        <item x="16"/>
+        <item x="88"/>
+        <item x="160"/>
+        <item x="232"/>
+        <item x="22"/>
+        <item x="94"/>
+        <item x="166"/>
+        <item x="238"/>
+        <item x="28"/>
+        <item x="100"/>
+        <item x="172"/>
+        <item x="244"/>
+        <item x="34"/>
+        <item x="106"/>
+        <item x="178"/>
+        <item x="40"/>
+        <item x="112"/>
+        <item x="184"/>
+        <item x="46"/>
+        <item x="118"/>
+        <item x="190"/>
+        <item x="52"/>
+        <item x="124"/>
+        <item x="196"/>
+        <item x="58"/>
+        <item x="130"/>
+        <item x="202"/>
+        <item x="64"/>
+        <item x="136"/>
+        <item x="208"/>
+        <item x="0"/>
+        <item x="71"/>
+        <item x="143"/>
+        <item x="215"/>
+        <item x="6"/>
+        <item x="77"/>
+        <item x="149"/>
+        <item x="221"/>
+        <item x="11"/>
+        <item x="83"/>
+        <item x="155"/>
+        <item x="227"/>
+        <item x="17"/>
+        <item x="89"/>
+        <item x="161"/>
+        <item x="233"/>
+        <item x="23"/>
+        <item x="95"/>
+        <item x="167"/>
+        <item x="239"/>
+        <item x="29"/>
+        <item x="101"/>
+        <item x="173"/>
+        <item x="245"/>
+        <item x="35"/>
+        <item x="107"/>
+        <item x="179"/>
+        <item x="41"/>
+        <item x="113"/>
+        <item x="185"/>
+        <item x="47"/>
+        <item x="119"/>
+        <item x="191"/>
+        <item x="53"/>
+        <item x="125"/>
+        <item x="197"/>
+        <item x="59"/>
+        <item x="131"/>
+        <item x="203"/>
+        <item x="65"/>
+        <item x="137"/>
+        <item x="209"/>
+        <item x="1"/>
+        <item x="72"/>
+        <item x="144"/>
+        <item x="216"/>
+        <item x="7"/>
+        <item x="78"/>
+        <item x="150"/>
+        <item x="222"/>
+        <item x="12"/>
+        <item x="84"/>
+        <item x="156"/>
+        <item x="228"/>
+        <item x="18"/>
+        <item x="90"/>
+        <item x="162"/>
+        <item x="234"/>
+        <item x="24"/>
+        <item x="96"/>
+        <item x="168"/>
+        <item x="240"/>
+        <item x="30"/>
+        <item x="102"/>
+        <item x="174"/>
+        <item x="246"/>
+        <item x="36"/>
+        <item x="108"/>
+        <item x="180"/>
+        <item x="42"/>
+        <item x="114"/>
+        <item x="186"/>
+        <item x="48"/>
+        <item x="120"/>
+        <item x="192"/>
+        <item x="54"/>
+        <item x="126"/>
+        <item x="198"/>
+        <item x="60"/>
+        <item x="132"/>
+        <item x="204"/>
+        <item x="66"/>
+        <item x="138"/>
+        <item x="210"/>
+        <item x="2"/>
+        <item x="73"/>
+        <item x="145"/>
+        <item x="217"/>
+        <item x="8"/>
+        <item x="79"/>
+        <item x="151"/>
+        <item x="223"/>
+        <item x="13"/>
+        <item x="85"/>
+        <item x="157"/>
+        <item x="229"/>
+        <item x="19"/>
+        <item x="91"/>
+        <item x="163"/>
+        <item x="235"/>
+        <item x="25"/>
+        <item x="97"/>
+        <item x="169"/>
+        <item x="241"/>
+        <item x="31"/>
+        <item x="103"/>
+        <item x="175"/>
+        <item x="247"/>
+        <item x="37"/>
+        <item x="109"/>
+        <item x="181"/>
+        <item x="43"/>
+        <item x="115"/>
+        <item x="187"/>
+        <item x="49"/>
+        <item x="121"/>
+        <item x="193"/>
+        <item x="55"/>
+        <item x="127"/>
+        <item x="199"/>
+        <item x="61"/>
+        <item x="133"/>
+        <item x="205"/>
+        <item x="67"/>
+        <item x="139"/>
+        <item x="211"/>
+        <item x="3"/>
+        <item x="74"/>
+        <item x="146"/>
+        <item x="218"/>
+        <item x="9"/>
+        <item x="80"/>
+        <item x="152"/>
+        <item x="224"/>
+        <item x="14"/>
+        <item x="86"/>
+        <item x="158"/>
+        <item x="230"/>
+        <item x="20"/>
+        <item x="92"/>
+        <item x="164"/>
+        <item x="236"/>
+        <item x="26"/>
+        <item x="98"/>
+        <item x="170"/>
+        <item x="242"/>
+        <item x="32"/>
+        <item x="104"/>
+        <item x="176"/>
+        <item x="248"/>
+        <item x="38"/>
+        <item x="110"/>
+        <item x="182"/>
+        <item x="44"/>
+        <item x="116"/>
+        <item x="188"/>
+        <item x="50"/>
+        <item x="122"/>
+        <item x="194"/>
+        <item x="56"/>
+        <item x="128"/>
+        <item x="200"/>
+        <item x="62"/>
+        <item x="134"/>
+        <item x="206"/>
+        <item x="68"/>
+        <item x="140"/>
+        <item x="212"/>
+        <item x="4"/>
+        <item x="75"/>
+        <item x="147"/>
+        <item x="219"/>
+        <item x="81"/>
+        <item x="153"/>
+        <item x="225"/>
+        <item x="15"/>
+        <item x="87"/>
+        <item x="159"/>
+        <item x="231"/>
+        <item x="21"/>
+        <item x="93"/>
+        <item x="165"/>
+        <item x="237"/>
+        <item x="27"/>
+        <item x="99"/>
+        <item x="171"/>
+        <item x="243"/>
+        <item x="33"/>
+        <item x="105"/>
+        <item x="177"/>
+        <item x="249"/>
+        <item x="39"/>
+        <item x="111"/>
+        <item x="183"/>
+        <item x="45"/>
+        <item x="117"/>
+        <item x="189"/>
+        <item x="51"/>
+        <item x="123"/>
+        <item x="195"/>
+        <item x="57"/>
+        <item x="129"/>
+        <item x="201"/>
+        <item x="63"/>
+        <item x="135"/>
+        <item x="207"/>
+        <item x="69"/>
+        <item x="141"/>
+        <item x="213"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of BookingID" fld="0" subtotal="count" baseField="5" baseItem="1"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="8" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_RoomNo" xr10:uid="{FC762340-3809-4E26-9D63-7D14763AE321}" sourceName="RoomNo">
   <pivotTables>
@@ -12415,7 +12509,7 @@
       <c r="A4" s="4">
         <v>201</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>379769</v>
       </c>
     </row>
@@ -12423,7 +12517,7 @@
       <c r="A5" s="4">
         <v>202</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>332367</v>
       </c>
     </row>
@@ -12431,7 +12525,7 @@
       <c r="A6" s="4">
         <v>203</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>484569</v>
       </c>
     </row>
@@ -12439,7 +12533,7 @@
       <c r="A7" s="4">
         <v>204</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7">
         <v>566865</v>
       </c>
     </row>
@@ -12447,7 +12541,7 @@
       <c r="A8" s="4">
         <v>205</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8">
         <v>226497</v>
       </c>
     </row>
@@ -12455,7 +12549,7 @@
       <c r="A9" s="4">
         <v>206</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9">
         <v>845859</v>
       </c>
     </row>
@@ -12463,7 +12557,7 @@
       <c r="A10" s="4" t="s">
         <v>903</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10">
         <v>2835926</v>
       </c>
     </row>
@@ -12479,7 +12573,7 @@
       <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15">
         <v>162</v>
       </c>
     </row>
@@ -12487,7 +12581,7 @@
       <c r="A16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16">
         <v>88</v>
       </c>
     </row>
@@ -12495,7 +12589,7 @@
       <c r="A17" s="4" t="s">
         <v>903</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17">
         <v>250</v>
       </c>
     </row>
@@ -12511,7 +12605,7 @@
       <c r="A44" s="4">
         <v>201</v>
       </c>
-      <c r="B44" s="5">
+      <c r="B44">
         <v>43</v>
       </c>
     </row>
@@ -12519,7 +12613,7 @@
       <c r="A45" s="4">
         <v>202</v>
       </c>
-      <c r="B45" s="5">
+      <c r="B45">
         <v>41</v>
       </c>
     </row>
@@ -12527,7 +12621,7 @@
       <c r="A46" s="4">
         <v>203</v>
       </c>
-      <c r="B46" s="5">
+      <c r="B46">
         <v>42</v>
       </c>
     </row>
@@ -12535,7 +12629,7 @@
       <c r="A47" s="4">
         <v>204</v>
       </c>
-      <c r="B47" s="5">
+      <c r="B47">
         <v>41</v>
       </c>
     </row>
@@ -12543,7 +12637,7 @@
       <c r="A48" s="4">
         <v>205</v>
       </c>
-      <c r="B48" s="5">
+      <c r="B48">
         <v>42</v>
       </c>
     </row>
@@ -12551,7 +12645,7 @@
       <c r="A49" s="4">
         <v>206</v>
       </c>
-      <c r="B49" s="5">
+      <c r="B49">
         <v>41</v>
       </c>
     </row>
@@ -12559,7 +12653,7 @@
       <c r="A50" s="4" t="s">
         <v>903</v>
       </c>
-      <c r="B50" s="5">
+      <c r="B50">
         <v>250</v>
       </c>
     </row>
@@ -12575,7 +12669,7 @@
       <c r="A68" s="4">
         <v>2</v>
       </c>
-      <c r="B68" s="5">
+      <c r="B68">
         <v>171</v>
       </c>
     </row>
@@ -12583,7 +12677,7 @@
       <c r="A69" s="4">
         <v>3</v>
       </c>
-      <c r="B69" s="5">
+      <c r="B69">
         <v>43</v>
       </c>
     </row>
@@ -12591,7 +12685,7 @@
       <c r="A70" s="4">
         <v>4</v>
       </c>
-      <c r="B70" s="5">
+      <c r="B70">
         <v>36</v>
       </c>
     </row>
@@ -12599,7 +12693,7 @@
       <c r="A71" s="4" t="s">
         <v>903</v>
       </c>
-      <c r="B71" s="5">
+      <c r="B71">
         <v>250</v>
       </c>
     </row>
@@ -19930,50 +20024,50 @@
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:19" ht="20" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>906</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
     </row>
     <row r="2" spans="1:19" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>907</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -19995,13 +20089,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="5" t="s">
         <v>908</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="5" t="s">
         <v>909</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="5" t="s">
         <v>910</v>
       </c>
     </row>

</xml_diff>